<commit_message>
chore: daily development snapshot 2026-09-21
</commit_message>
<xml_diff>
--- a/docs/开房规则表/牛牛/全国牛牛.xlsx
+++ b/docs/开房规则表/牛牛/全国牛牛.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公共创建规则" sheetId="1" r:id="R6ff03a98c90542b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公共创建规则" sheetId="1" r:id="R48429bb1b01a416b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1120,12 +1120,8 @@
       <x:c r="F2"/>
     </x:row>
     <x:row r="3" s="1" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A3" s="2" t="str">
-        <x:v>游戏名称</x:v>
-      </x:c>
-      <x:c r="B3" s="3" t="str">
-        <x:v>牛牛</x:v>
-      </x:c>
+      <x:c r="A3" s="2"/>
+      <x:c r="B3" s="3"/>
       <x:c r="C3"/>
       <x:c r="D3"/>
       <x:c r="E3"/>
@@ -1144,9 +1140,7 @@
       <x:c r="F4"/>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A5" t="str">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="A5"/>
       <x:c r="B5" t="str">
         <x:v>98</x:v>
       </x:c>

</xml_diff>